<commit_message>
Changed and cleaned example files
</commit_message>
<xml_diff>
--- a/output/multiple_solutions.xlsx
+++ b/output/multiple_solutions.xlsx
@@ -32,6 +32,9 @@
     <t xml:space="preserve">pref4</t>
   </si>
   <si>
+    <t xml:space="preserve">pref5</t>
+  </si>
+  <si>
     <t xml:space="preserve">Anna</t>
   </si>
   <si>
@@ -66,9 +69,6 @@
   </si>
   <si>
     <t xml:space="preserve">solution_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">solution_3</t>
   </si>
 </sst>
 </file>
@@ -418,10 +418,13 @@
       <c r="E2" t="s">
         <v>5</v>
       </c>
+      <c r="F2" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" t="n">
         <v>3</v>
@@ -431,10 +434,11 @@
       </c>
       <c r="D3"/>
       <c r="E3"/>
+      <c r="F3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B4" t="n">
         <v>2</v>
@@ -446,10 +450,11 @@
         <v>1</v>
       </c>
       <c r="E4"/>
+      <c r="F4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" t="n">
         <v>3</v>
@@ -459,10 +464,11 @@
       </c>
       <c r="D5"/>
       <c r="E5"/>
+      <c r="F5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" t="n">
         <v>4</v>
@@ -474,27 +480,29 @@
         <v>3</v>
       </c>
       <c r="E6"/>
+      <c r="F6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7" t="n">
         <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="F7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B8" t="n">
         <v>3</v>
@@ -508,10 +516,11 @@
       <c r="E8" t="n">
         <v>2</v>
       </c>
+      <c r="F8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B9" t="n">
         <v>1</v>
@@ -525,10 +534,11 @@
       <c r="E9" t="n">
         <v>4</v>
       </c>
+      <c r="F9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B10" t="n">
         <v>3</v>
@@ -538,15 +548,13 @@
       </c>
       <c r="D10"/>
       <c r="E10"/>
+      <c r="F10"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E13" t="s">
-        <v>17</v>
-      </c>
-      <c r="I13" t="s">
         <v>18</v>
       </c>
     </row>
@@ -555,33 +563,24 @@
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C14" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" t="s">
+        <v>1</v>
+      </c>
+      <c r="F14" t="s">
         <v>16</v>
       </c>
-      <c r="E14" t="s">
-        <v>1</v>
-      </c>
-      <c r="F14" t="s">
-        <v>15</v>
-      </c>
       <c r="G14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I14" t="s">
-        <v>1</v>
-      </c>
-      <c r="J14" t="s">
-        <v>15</v>
-      </c>
-      <c r="K14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B15" t="n">
         <v>3</v>
@@ -590,56 +589,38 @@
         <v>4</v>
       </c>
       <c r="E15" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F15" t="n">
         <v>3</v>
       </c>
       <c r="G15" t="n">
-        <v>4</v>
-      </c>
-      <c r="I15" t="s">
-        <v>6</v>
-      </c>
-      <c r="J15" t="n">
-        <v>3</v>
-      </c>
-      <c r="K15" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
         <v>5</v>
       </c>
       <c r="E16" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F16" t="n">
         <v>2</v>
       </c>
       <c r="G16" t="n">
-        <v>5</v>
-      </c>
-      <c r="I16" t="s">
-        <v>7</v>
-      </c>
-      <c r="J16" t="n">
-        <v>1</v>
-      </c>
-      <c r="K16" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B17" t="n">
         <v>2</v>
@@ -648,27 +629,18 @@
         <v>3</v>
       </c>
       <c r="E17" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F17" t="n">
         <v>2</v>
       </c>
       <c r="G17" t="n">
-        <v>3</v>
-      </c>
-      <c r="I17" t="s">
-        <v>8</v>
-      </c>
-      <c r="J17" t="n">
-        <v>2</v>
-      </c>
-      <c r="K17" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B18" t="n">
         <v>1</v>
@@ -677,27 +649,18 @@
         <v>4</v>
       </c>
       <c r="E18" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F18" t="n">
         <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>4</v>
-      </c>
-      <c r="I18" t="s">
-        <v>9</v>
-      </c>
-      <c r="J18" t="n">
-        <v>1</v>
-      </c>
-      <c r="K18" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B19" t="n">
         <v>2</v>
@@ -706,56 +669,38 @@
         <v>5</v>
       </c>
       <c r="E19" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19" t="n">
-        <v>5</v>
-      </c>
-      <c r="I19" t="s">
-        <v>10</v>
-      </c>
-      <c r="J19" t="n">
-        <v>2</v>
-      </c>
-      <c r="K19" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C20" t="n">
         <v>5</v>
       </c>
       <c r="E20" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>5</v>
-      </c>
-      <c r="I20" t="s">
-        <v>11</v>
-      </c>
-      <c r="J20" t="n">
-        <v>3</v>
-      </c>
-      <c r="K20" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B21" t="n">
         <v>1</v>
@@ -764,27 +709,18 @@
         <v>2</v>
       </c>
       <c r="E21" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>2</v>
-      </c>
-      <c r="I21" t="s">
-        <v>12</v>
-      </c>
-      <c r="J21" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B22" t="n">
         <v>3</v>
@@ -793,21 +729,12 @@
         <v>4</v>
       </c>
       <c r="E22" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F22" t="n">
         <v>3</v>
       </c>
       <c r="G22" t="n">
-        <v>4</v>
-      </c>
-      <c r="I22" t="s">
-        <v>13</v>
-      </c>
-      <c r="J22" t="n">
-        <v>3</v>
-      </c>
-      <c r="K22" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>